<commit_message>
Fix corporate action duplicates, ticker mismatches, and missing manual corrections
- corporate_actions.bean: remove duplicate WEGE3 desdobramento (was
  applying 2x ratio, inflating holdings 4x instead of 2x); fix EGIE3
  bonificacao ratio 1.1 -> 1.4 (Yahoo listed event twice, reconcile
  picked wrong one; broker confirms 620 shares = 1.4 ratio)
- transactions.bean: fix IRIM15 -> IRIM11 (importer misclassification),
  shorten CDB-CDB526CSFDK-BANCO-DO-BRASIL-S-A -> CDB-CDB526CSFDK to
  match buy entry ticker, remove unmatched CVCB11 transfer, adjust
  WEGE3 buy 400@9.15 -> 200@18.30 (pre-split quantity correction)
- prices/prices.bean: remove MALL11.bean include (file never generated,
  ticker delisted)
- manual_corrections.bean: add subscricao entries, IRDM11->IRIM11
  merger conversion entry, fix MCCI11 subscricao cash amount
- main.bean: include manual_corrections.bean
</commit_message>
<xml_diff>
--- a/export_backlog/negociacao-2019.xlsx
+++ b/export_backlog/negociacao-2019.xlsx
@@ -94,6 +94,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -121,6 +122,7 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -165,32 +167,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -333,392 +339,392 @@
   <dimension ref="A1:J1048576"/>
   <sheetFormatPr defaultColWidth="9.7578125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26.49"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="25.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="31.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="0" width="35.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="31.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="26.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="31.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="35.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>43684</v>
       </c>
-      <c r="B2" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="3" t="n">
+      <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="H2" s="5" t="n">
         <v>25.2</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="5" t="n">
         <v>2523.44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>43682</v>
       </c>
-      <c r="B3" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="3" t="n">
+      <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="H3" s="5" t="n">
         <v>25.6</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I3" s="5" t="n">
         <v>2563.47</v>
       </c>
-      <c r="J3" s="5"/>
+      <c r="J3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>43682</v>
       </c>
-      <c r="B4" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="3" t="n">
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="5" t="n">
         <v>25.8</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="5" t="n">
         <v>2583.47</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>43661</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="3" t="n">
+      <c r="C5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="4" t="n">
         <v>94</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="5" t="n">
         <v>28.44</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="5" t="n">
         <v>2670.56</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="3" t="n">
         <v>43661</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="3" t="n">
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H6" s="5" t="n">
         <v>28.43</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="5" t="n">
         <v>27.73</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="3" t="n">
         <v>43656</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="3" t="n">
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="I7" s="5" t="n">
         <v>5576.43</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="3" t="n">
         <v>43570</v>
       </c>
-      <c r="B8" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="3" t="n">
+      <c r="B8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="4" t="n">
         <v>95</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="H8" s="5" t="n">
         <v>25.87</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="I8" s="5" t="n">
         <v>2461.14</v>
       </c>
-      <c r="J8" s="5"/>
+      <c r="J8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="3" t="n">
         <v>43543</v>
       </c>
-      <c r="B9" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="0" t="s">
+      <c r="B9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="G9" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="H9" s="5" t="n">
         <v>43.2</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="I9" s="5" t="n">
         <v>4323.68</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="3" t="n">
         <v>43543</v>
       </c>
-      <c r="B10" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="0" t="s">
+      <c r="B10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="G10" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="H10" s="5" t="n">
         <v>31.82</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="I10" s="5" t="n">
         <v>3185.68</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="3" t="n">
         <v>43391</v>
       </c>
-      <c r="B11" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="0" t="s">
+      <c r="B11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="3" t="n">
-        <v>400</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>9.15</v>
-      </c>
-      <c r="I11" s="4" t="n">
+      <c r="G11" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="I11" s="5" t="n">
         <v>3682.63</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="3" t="n">
         <v>43258</v>
       </c>
-      <c r="B12" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="3" t="n">
+      <c r="B12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="H12" s="5" t="n">
         <v>15.5</v>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="I12" s="5" t="n">
         <v>1571.93</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="n">
+      <c r="A13" s="3" t="n">
         <v>43248</v>
       </c>
-      <c r="B13" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="3" t="n">
+      <c r="B13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="H13" s="5" t="n">
         <v>17.6</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="I13" s="5" t="n">
         <v>1782.01</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="6"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="7"/>
     </row>
     <row r="1048539" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048540" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>